<commit_message>
Switch overlay line from visit_id to browse_id
visit_id is per-session so it's tautologically near-unique vs scans.
browse_id is the persistent browser cookie, which actually answers
"how many different people scanned" — 163 distinct browsers behind
the 175 scans; 11 of them came back to scan a second time.

https://claude.ai/code/session_01PM89wz7vnfvW2NRaFUoooy
</commit_message>
<xml_diff>
--- a/qr_weekly_with_visits.xlsx
+++ b/qr_weekly_with_visits.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Distinct visits</t>
+          <t>Distinct browsers</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
         <v>10</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -735,7 +735,7 @@
         <v>16</v>
       </c>
       <c r="C11" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -826,7 +826,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
@@ -852,7 +852,7 @@
         <v>12</v>
       </c>
       <c r="C20" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>